<commit_message>
having trouble with tibbles
</commit_message>
<xml_diff>
--- a/inst/extdata/Antigen 2 - info sheet.xlsx
+++ b/inst/extdata/Antigen 2 - info sheet.xlsx
@@ -831,7 +831,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:S168"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.35"/>
@@ -2895,7 +2895,7 @@
         <v>71</v>
       </c>
       <c r="M35" s="0" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="N35" s="0" t="s">
         <v>26</v>
@@ -2913,7 +2913,7 @@
         <v>26</v>
       </c>
       <c r="S35" s="0" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>